<commit_message>
...the hex display was the wrong way around
</commit_message>
<xml_diff>
--- a/8Bit Computer ver2.0/excel/commands.xlsx
+++ b/8Bit Computer ver2.0/excel/commands.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Files\GitHub\Private\Computer_HTL\8Bit Computer ver2.0\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Files\GitHub\Computer_HTL\8Bit Computer ver2.0\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6BD9E6C-90AF-4050-A7B1-7BEE78D0463B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B6D5AF-3B89-4E6F-B57C-315EDBEE55A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38295" yWindow="10905" windowWidth="16410" windowHeight="14145" xr2:uid="{3256ACAE-F419-450F-8F49-2183F1DCCADE}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="146">
   <si>
     <t>NOP</t>
   </si>
@@ -461,6 +461,9 @@
   </si>
   <si>
     <t>LOAD DISTANCE</t>
+  </si>
+  <si>
+    <t>Tested</t>
   </si>
 </sst>
 </file>
@@ -726,7 +729,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -837,6 +840,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1173,26 +1182,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02BDFC33-BE10-4835-94A0-E5C8BC037442}">
-  <dimension ref="A1:AH72"/>
+  <dimension ref="A1:AI72"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
     <col min="2" max="2" width="41.42578125" customWidth="1"/>
     <col min="3" max="3" width="8.42578125" customWidth="1"/>
     <col min="4" max="5" width="12.140625" customWidth="1"/>
-    <col min="6" max="6" width="7.28515625" customWidth="1"/>
-    <col min="7" max="7" width="7.140625" customWidth="1"/>
-    <col min="8" max="8" width="7.42578125" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" customWidth="1"/>
-    <col min="10" max="10" width="9" customWidth="1"/>
-    <col min="11" max="11" width="10.85546875" customWidth="1"/>
-    <col min="12" max="12" width="9" customWidth="1"/>
-    <col min="13" max="13" width="10" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" customWidth="1"/>
-    <col min="17" max="17" width="67.7109375" customWidth="1"/>
+    <col min="6" max="6" width="6.7109375" customWidth="1"/>
+    <col min="7" max="7" width="7.28515625" customWidth="1"/>
+    <col min="8" max="8" width="7.140625" customWidth="1"/>
+    <col min="9" max="9" width="7.42578125" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" customWidth="1"/>
+    <col min="11" max="11" width="9" customWidth="1"/>
+    <col min="12" max="12" width="10.85546875" customWidth="1"/>
+    <col min="13" max="13" width="9" customWidth="1"/>
+    <col min="14" max="14" width="10" customWidth="1"/>
+    <col min="15" max="15" width="9.7109375" customWidth="1"/>
+    <col min="18" max="18" width="67.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="1" customFormat="1" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" s="1" customFormat="1" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="40" t="s">
         <v>36</v>
       </c>
@@ -1207,37 +1217,40 @@
         <v>30</v>
       </c>
       <c r="F1" s="16" t="s">
+        <v>145</v>
+      </c>
+      <c r="G1" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="H1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="I1" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="J1" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="J1" s="16" t="s">
+      <c r="K1" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="K1" s="16" t="s">
+      <c r="L1" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="16" t="s">
+      <c r="M1" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="N1" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="O1" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="O1" s="17" t="s">
+      <c r="P1" s="17" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1249,21 +1262,22 @@
       </c>
       <c r="D2" s="28"/>
       <c r="E2" s="29"/>
-      <c r="F2" s="30"/>
+      <c r="F2" s="44"/>
       <c r="G2" s="30"/>
       <c r="H2" s="30"/>
       <c r="I2" s="30"/>
       <c r="J2" s="30"/>
-      <c r="K2" s="29"/>
+      <c r="K2" s="30"/>
       <c r="L2" s="29"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="31"/>
+      <c r="M2" s="29"/>
+      <c r="N2" s="30"/>
       <c r="O2" s="31"/>
-      <c r="Q2" s="35" t="s">
+      <c r="P2" s="31"/>
+      <c r="R2" s="35" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B3" s="9" t="s">
         <v>59</v>
       </c>
@@ -1274,25 +1288,26 @@
       <c r="E3" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="6"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
-      <c r="I3" s="4"/>
+      <c r="I3" s="6"/>
       <c r="J3" s="4"/>
-      <c r="K3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="L3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="M3" s="4"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q3" s="36" t="s">
+      <c r="N3" s="4"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="R3" s="36" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="9" t="s">
         <v>58</v>
       </c>
@@ -1305,27 +1320,28 @@
       <c r="E4" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="F4" s="6"/>
+      <c r="F4" s="44"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
-      <c r="I4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="L4" s="4"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="M4" s="4"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q4" s="37" t="s">
+      <c r="N4" s="4"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="R4" s="37" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>127</v>
       </c>
@@ -1339,21 +1355,22 @@
         <v>33</v>
       </c>
       <c r="E5" s="34"/>
-      <c r="F5" s="7"/>
+      <c r="F5" s="44"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
-      <c r="I5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J5" s="2"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="2"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K5" s="2"/>
+      <c r="L5" s="1"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
-      <c r="O5" s="1"/>
-      <c r="Q5" s="1"/>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O5" s="2"/>
+      <c r="P5" s="1"/>
+      <c r="R5" s="1"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B6" s="15" t="s">
         <v>114</v>
       </c>
@@ -1364,21 +1381,22 @@
         <v>33</v>
       </c>
       <c r="E6" s="34"/>
-      <c r="F6" s="6"/>
+      <c r="F6" s="44"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
-      <c r="I6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J6" s="2"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="2"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K6" s="2"/>
+      <c r="L6" s="1"/>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
-      <c r="O6" s="1"/>
-      <c r="Q6" s="1"/>
-    </row>
-    <row r="7" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="O6" s="2"/>
+      <c r="P6" s="1"/>
+      <c r="R6" s="1"/>
+    </row>
+    <row r="7" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="19"/>
       <c r="B7" s="20" t="s">
         <v>115</v>
@@ -1390,21 +1408,22 @@
       <c r="E7" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="F7" s="6"/>
+      <c r="F7" s="44"/>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="M7" s="2"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="N7" s="2"/>
-      <c r="O7" s="1"/>
-      <c r="Q7" s="1"/>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O7" s="2"/>
+      <c r="P7" s="1"/>
+      <c r="R7" s="1"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>37</v>
       </c>
@@ -1420,21 +1439,22 @@
       <c r="E8" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="6"/>
+      <c r="F8" s="44"/>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
-      <c r="I8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="J8" s="4"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
       <c r="M8" s="4"/>
-      <c r="N8" s="5"/>
+      <c r="N8" s="4"/>
       <c r="O8" s="5"/>
-      <c r="Q8" s="1"/>
-    </row>
-    <row r="9" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P8" s="5"/>
+      <c r="R8" s="1"/>
+    </row>
+    <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="15" t="s">
         <v>38</v>
       </c>
@@ -1447,21 +1467,22 @@
       <c r="E9" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="6"/>
+      <c r="F9" s="44"/>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="K9" s="4"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
-      <c r="N9" s="5"/>
+      <c r="N9" s="4"/>
       <c r="O9" s="5"/>
-      <c r="Q9" s="1"/>
-    </row>
-    <row r="10" spans="1:17" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P9" s="5"/>
+      <c r="R9" s="1"/>
+    </row>
+    <row r="10" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="38" t="s">
         <v>35</v>
       </c>
@@ -1476,38 +1497,41 @@
         <v>30</v>
       </c>
       <c r="F10" s="16" t="s">
+        <v>145</v>
+      </c>
+      <c r="G10" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="G10" s="16" t="s">
+      <c r="H10" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="H10" s="16" t="s">
+      <c r="I10" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="I10" s="16" t="s">
+      <c r="J10" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="J10" s="16" t="s">
+      <c r="K10" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="K10" s="16" t="s">
+      <c r="L10" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="L10" s="16" t="s">
+      <c r="M10" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="M10" s="16" t="s">
+      <c r="N10" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="N10" s="16" t="s">
+      <c r="O10" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="O10" s="17" t="s">
+      <c r="P10" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="Q10" s="1"/>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R10" s="1"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -1521,27 +1545,28 @@
         <v>136</v>
       </c>
       <c r="E11" s="29"/>
-      <c r="F11" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F11" s="44"/>
       <c r="G11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H11" s="2"/>
+      <c r="H11" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="I11" s="2"/>
-      <c r="J11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K11" s="4"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L11" s="4"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O11" s="8"/>
-      <c r="Q11" s="1"/>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="M11" s="4"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="P11" s="8"/>
+      <c r="R11" s="1"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B12" s="9" t="s">
         <v>31</v>
       </c>
@@ -1552,29 +1577,30 @@
         <v>136</v>
       </c>
       <c r="E12" s="29"/>
-      <c r="F12" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F12" s="44"/>
       <c r="G12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H12" s="2"/>
+      <c r="H12" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="I12" s="2"/>
-      <c r="J12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K12" s="4"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L12" s="4"/>
-      <c r="M12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="N12" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O12" s="8"/>
-      <c r="Q12" s="1"/>
-    </row>
-    <row r="13" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M12" s="4"/>
+      <c r="N12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="O12" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="P12" s="8"/>
+      <c r="R12" s="1"/>
+    </row>
+    <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="9" t="s">
         <v>5</v>
       </c>
@@ -1585,29 +1611,30 @@
         <v>136</v>
       </c>
       <c r="E13" s="29"/>
-      <c r="F13" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F13" s="44"/>
       <c r="G13" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="2"/>
+      <c r="H13" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="I13" s="2"/>
-      <c r="J13" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K13" s="4"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L13" s="4"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O13" s="8"/>
-      <c r="Q13" s="1" t="s">
+      <c r="M13" s="4"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="P13" s="8"/>
+      <c r="R13" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
         <v>40</v>
       </c>
@@ -1621,25 +1648,26 @@
         <v>136</v>
       </c>
       <c r="E14" s="29"/>
-      <c r="F14" s="2"/>
+      <c r="F14" s="44"/>
       <c r="G14" s="2"/>
-      <c r="H14" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2" t="s">
+      <c r="H14" s="2"/>
+      <c r="I14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="K14" s="4"/>
       <c r="L14" s="4"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O14" s="8"/>
-      <c r="Q14" s="1"/>
-    </row>
-    <row r="15" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M14" s="4"/>
+      <c r="N14" s="2"/>
+      <c r="O14" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="P14" s="8"/>
+      <c r="R14" s="1"/>
+    </row>
+    <row r="15" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="10" t="s">
         <v>7</v>
       </c>
@@ -1650,27 +1678,28 @@
         <v>136</v>
       </c>
       <c r="E15" s="29"/>
-      <c r="F15" s="2"/>
+      <c r="F15" s="44"/>
       <c r="G15" s="2"/>
-      <c r="H15" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2" t="s">
+      <c r="H15" s="2"/>
+      <c r="I15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="K15" s="4"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O15" s="8"/>
-      <c r="Q15" s="1" t="s">
+      <c r="M15" s="4"/>
+      <c r="N15" s="2"/>
+      <c r="O15" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="P15" s="8"/>
+      <c r="R15" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
         <v>3</v>
       </c>
@@ -1684,25 +1713,26 @@
         <v>137</v>
       </c>
       <c r="E16" s="29"/>
-      <c r="F16" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G16" s="2"/>
+      <c r="F16" s="44"/>
+      <c r="G16" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K16" s="4"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L16" s="4"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="3"/>
-      <c r="O16" s="8"/>
-      <c r="Q16" s="1" t="s">
+      <c r="M16" s="4"/>
+      <c r="N16" s="2"/>
+      <c r="O16" s="3"/>
+      <c r="P16" s="8"/>
+      <c r="R16" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B17" s="9" t="s">
         <v>22</v>
       </c>
@@ -1713,25 +1743,26 @@
         <v>137</v>
       </c>
       <c r="E17" s="29"/>
-      <c r="F17" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F17" s="44"/>
       <c r="G17" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H17" s="2"/>
+      <c r="H17" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="I17" s="2"/>
-      <c r="J17" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K17" s="4"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L17" s="4"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="3"/>
-      <c r="O17" s="8"/>
-      <c r="Q17" s="1"/>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="M17" s="4"/>
+      <c r="N17" s="2"/>
+      <c r="O17" s="3"/>
+      <c r="P17" s="8"/>
+      <c r="R17" s="1"/>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B18" s="9" t="s">
         <v>23</v>
       </c>
@@ -1742,27 +1773,28 @@
         <v>137</v>
       </c>
       <c r="E18" s="29"/>
-      <c r="F18" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F18" s="44"/>
       <c r="G18" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H18" s="2"/>
+      <c r="H18" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="I18" s="2"/>
-      <c r="J18" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K18" s="4"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L18" s="4"/>
-      <c r="M18" s="2"/>
-      <c r="N18" s="3"/>
-      <c r="O18" s="8"/>
-      <c r="Q18" s="1" t="s">
+      <c r="M18" s="4"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="3"/>
+      <c r="P18" s="8"/>
+      <c r="R18" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B19" s="9" t="s">
         <v>24</v>
       </c>
@@ -1773,27 +1805,28 @@
         <v>137</v>
       </c>
       <c r="E19" s="29"/>
-      <c r="F19" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F19" s="44"/>
       <c r="G19" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H19" s="2"/>
+      <c r="H19" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="I19" s="2"/>
-      <c r="J19" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K19" s="4"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L19" s="4"/>
-      <c r="M19" s="2"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="8"/>
-      <c r="Q19" s="1" t="s">
+      <c r="M19" s="4"/>
+      <c r="N19" s="2"/>
+      <c r="O19" s="3"/>
+      <c r="P19" s="8"/>
+      <c r="R19" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B20" s="9" t="s">
         <v>25</v>
       </c>
@@ -1804,25 +1837,26 @@
         <v>137</v>
       </c>
       <c r="E20" s="29"/>
-      <c r="F20" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G20" s="2"/>
+      <c r="F20" s="44"/>
+      <c r="G20" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
-      <c r="J20" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K20" s="4"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L20" s="4"/>
-      <c r="M20" s="2"/>
-      <c r="N20" s="3"/>
-      <c r="O20" s="8"/>
-      <c r="Q20" s="1" t="s">
+      <c r="M20" s="4"/>
+      <c r="N20" s="2"/>
+      <c r="O20" s="3"/>
+      <c r="P20" s="8"/>
+      <c r="R20" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B21" s="9" t="s">
         <v>26</v>
       </c>
@@ -1833,25 +1867,26 @@
         <v>137</v>
       </c>
       <c r="E21" s="29"/>
-      <c r="F21" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F21" s="44"/>
       <c r="G21" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H21" s="2"/>
+      <c r="H21" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="I21" s="2"/>
-      <c r="J21" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K21" s="4"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L21" s="4"/>
-      <c r="M21" s="2"/>
-      <c r="N21" s="3"/>
-      <c r="O21" s="8"/>
-      <c r="Q21" s="1"/>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="M21" s="4"/>
+      <c r="N21" s="2"/>
+      <c r="O21" s="3"/>
+      <c r="P21" s="8"/>
+      <c r="R21" s="1"/>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B22" s="9" t="s">
         <v>27</v>
       </c>
@@ -1862,27 +1897,28 @@
         <v>137</v>
       </c>
       <c r="E22" s="29"/>
-      <c r="F22" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F22" s="44"/>
       <c r="G22" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H22" s="2"/>
+      <c r="H22" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="I22" s="2"/>
-      <c r="J22" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K22" s="4"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L22" s="4"/>
-      <c r="M22" s="2"/>
-      <c r="N22" s="3"/>
-      <c r="O22" s="8"/>
-      <c r="Q22" s="1" t="s">
+      <c r="M22" s="4"/>
+      <c r="N22" s="2"/>
+      <c r="O22" s="3"/>
+      <c r="P22" s="8"/>
+      <c r="R22" s="1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="9" t="s">
         <v>28</v>
       </c>
@@ -1893,27 +1929,28 @@
         <v>137</v>
       </c>
       <c r="E23" s="29"/>
-      <c r="F23" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F23" s="44"/>
       <c r="G23" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H23" s="2"/>
+      <c r="H23" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="I23" s="2"/>
-      <c r="J23" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K23" s="4"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L23" s="4"/>
-      <c r="M23" s="2"/>
-      <c r="N23" s="3"/>
-      <c r="O23" s="8"/>
-      <c r="Q23" s="1" t="s">
+      <c r="M23" s="4"/>
+      <c r="N23" s="2"/>
+      <c r="O23" s="3"/>
+      <c r="P23" s="8"/>
+      <c r="R23" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
         <v>4</v>
       </c>
@@ -1927,26 +1964,27 @@
         <v>137</v>
       </c>
       <c r="E24" s="29"/>
-      <c r="F24" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F24" s="44"/>
       <c r="G24" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H24" s="2"/>
+      <c r="H24" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="I24" s="2"/>
-      <c r="J24" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K24" s="4"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L24" s="4"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O24" s="8"/>
-    </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="M24" s="4"/>
+      <c r="N24" s="2"/>
+      <c r="O24" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="P24" s="8"/>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B25" s="9" t="s">
         <v>47</v>
       </c>
@@ -1957,26 +1995,27 @@
         <v>137</v>
       </c>
       <c r="E25" s="29"/>
-      <c r="F25" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F25" s="44"/>
       <c r="G25" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H25" s="2"/>
+      <c r="H25" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="I25" s="2"/>
-      <c r="J25" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K25" s="4"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L25" s="4"/>
-      <c r="M25" s="2"/>
-      <c r="N25" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O25" s="8"/>
-    </row>
-    <row r="26" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M25" s="4"/>
+      <c r="N25" s="2"/>
+      <c r="O25" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="P25" s="8"/>
+    </row>
+    <row r="26" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="9" t="s">
         <v>49</v>
       </c>
@@ -1987,26 +2026,27 @@
         <v>137</v>
       </c>
       <c r="E26" s="29"/>
-      <c r="F26" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F26" s="44"/>
       <c r="G26" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H26" s="2"/>
+      <c r="H26" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="I26" s="2"/>
-      <c r="J26" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K26" s="4"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L26" s="4"/>
-      <c r="M26" s="2"/>
-      <c r="N26" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O26" s="8"/>
-    </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="M26" s="4"/>
+      <c r="N26" s="2"/>
+      <c r="O26" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="P26" s="8"/>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
         <v>112</v>
       </c>
@@ -2020,20 +2060,21 @@
         <v>33</v>
       </c>
       <c r="E27" s="29"/>
-      <c r="F27" s="2"/>
+      <c r="F27" s="44"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
-      <c r="I27" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J27" s="2"/>
-      <c r="K27" s="4"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K27" s="2"/>
       <c r="L27" s="4"/>
-      <c r="M27" s="2"/>
-      <c r="N27" s="3"/>
-      <c r="O27" s="8"/>
-    </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="M27" s="4"/>
+      <c r="N27" s="2"/>
+      <c r="O27" s="3"/>
+      <c r="P27" s="8"/>
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B28" s="9" t="s">
         <v>71</v>
       </c>
@@ -2044,22 +2085,23 @@
         <v>33</v>
       </c>
       <c r="E28" s="29"/>
-      <c r="F28" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G28" s="2"/>
+      <c r="F28" s="44"/>
+      <c r="G28" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
-      <c r="J28" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K28" s="4"/>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L28" s="4"/>
-      <c r="M28" s="2"/>
-      <c r="N28" s="3"/>
-      <c r="O28" s="8"/>
-    </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="M28" s="4"/>
+      <c r="N28" s="2"/>
+      <c r="O28" s="3"/>
+      <c r="P28" s="8"/>
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B29" s="9" t="s">
         <v>65</v>
       </c>
@@ -2070,22 +2112,23 @@
         <v>33</v>
       </c>
       <c r="E29" s="29"/>
-      <c r="F29" s="2"/>
+      <c r="F29" s="44"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
-      <c r="I29" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J29" s="2"/>
-      <c r="K29" s="4"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K29" s="2"/>
       <c r="L29" s="4"/>
-      <c r="M29" s="2"/>
-      <c r="N29" s="3"/>
-      <c r="O29" s="8"/>
-      <c r="T29" s="11"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="2"/>
+      <c r="O29" s="3"/>
+      <c r="P29" s="8"/>
       <c r="U29" s="11"/>
-    </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V29" s="11"/>
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B30" s="9" t="s">
         <v>72</v>
       </c>
@@ -2096,22 +2139,23 @@
         <v>33</v>
       </c>
       <c r="E30" s="29"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H30" s="2"/>
+      <c r="F30" s="44"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="I30" s="2"/>
-      <c r="J30" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K30" s="4"/>
+      <c r="J30" s="2"/>
+      <c r="K30" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L30" s="4"/>
-      <c r="M30" s="2"/>
-      <c r="N30" s="3"/>
-      <c r="O30" s="8"/>
-    </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="M30" s="4"/>
+      <c r="N30" s="2"/>
+      <c r="O30" s="3"/>
+      <c r="P30" s="8"/>
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B31" s="15" t="s">
         <v>63</v>
       </c>
@@ -2122,20 +2166,21 @@
         <v>33</v>
       </c>
       <c r="E31" s="29"/>
-      <c r="F31" s="2"/>
+      <c r="F31" s="44"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
-      <c r="I31" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J31" s="2"/>
-      <c r="K31" s="4"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K31" s="2"/>
       <c r="L31" s="4"/>
-      <c r="M31" s="2"/>
-      <c r="N31" s="3"/>
-      <c r="O31" s="8"/>
-    </row>
-    <row r="32" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M31" s="4"/>
+      <c r="N31" s="2"/>
+      <c r="O31" s="3"/>
+      <c r="P31" s="8"/>
+    </row>
+    <row r="32" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9" t="s">
         <v>69</v>
       </c>
@@ -2146,24 +2191,25 @@
         <v>33</v>
       </c>
       <c r="E32" s="29"/>
-      <c r="F32" s="2"/>
+      <c r="F32" s="44"/>
       <c r="G32" s="2"/>
-      <c r="H32" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K32" s="4"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L32" s="4"/>
-      <c r="M32" s="2"/>
-      <c r="N32" s="3"/>
-      <c r="O32" s="8"/>
-      <c r="T32" s="11"/>
+      <c r="M32" s="4"/>
+      <c r="N32" s="2"/>
+      <c r="O32" s="3"/>
+      <c r="P32" s="8"/>
       <c r="U32" s="11"/>
-    </row>
-    <row r="33" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="V32" s="11"/>
+    </row>
+    <row r="33" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
         <v>19</v>
       </c>
@@ -2177,22 +2223,23 @@
         <v>33</v>
       </c>
       <c r="E33" s="29"/>
-      <c r="F33" s="2"/>
+      <c r="F33" s="44"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
-      <c r="I33" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J33" s="2"/>
-      <c r="K33" s="4"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K33" s="2"/>
       <c r="L33" s="4"/>
-      <c r="M33" s="2"/>
-      <c r="N33" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O33" s="8"/>
-    </row>
-    <row r="34" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="M33" s="4"/>
+      <c r="N33" s="2"/>
+      <c r="O33" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="P33" s="8"/>
+    </row>
+    <row r="34" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B34" s="9" t="s">
         <v>67</v>
       </c>
@@ -2203,22 +2250,23 @@
         <v>131</v>
       </c>
       <c r="E34" s="29"/>
-      <c r="F34" s="2"/>
+      <c r="F34" s="44"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
-      <c r="J34" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K34" s="4"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L34" s="4"/>
-      <c r="M34" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="N34" s="3"/>
-      <c r="O34" s="8"/>
-    </row>
-    <row r="35" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="M34" s="4"/>
+      <c r="N34" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="O34" s="3"/>
+      <c r="P34" s="8"/>
+    </row>
+    <row r="35" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B35" s="9" t="s">
         <v>68</v>
       </c>
@@ -2229,21 +2277,21 @@
         <v>133</v>
       </c>
       <c r="E35" s="29"/>
-      <c r="F35" s="2"/>
+      <c r="F35" s="44"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
-      <c r="J35" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K35" s="4"/>
+      <c r="J35" s="2"/>
+      <c r="K35" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L35" s="4"/>
-      <c r="M35" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="N35" s="3"/>
-      <c r="O35" s="8"/>
-      <c r="W35" s="11"/>
+      <c r="M35" s="4"/>
+      <c r="N35" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="O35" s="3"/>
+      <c r="P35" s="8"/>
       <c r="X35" s="11"/>
       <c r="Y35" s="11"/>
       <c r="Z35" s="11"/>
@@ -2255,8 +2303,9 @@
       <c r="AF35" s="11"/>
       <c r="AG35" s="11"/>
       <c r="AH35" s="11"/>
-    </row>
-    <row r="36" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AI35" s="11"/>
+    </row>
+    <row r="36" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="9" t="s">
         <v>8</v>
       </c>
@@ -2267,21 +2316,21 @@
         <v>134</v>
       </c>
       <c r="E36" s="29"/>
-      <c r="F36" s="2"/>
+      <c r="F36" s="44"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
-      <c r="J36" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K36" s="4"/>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L36" s="4"/>
-      <c r="M36" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="N36" s="3"/>
-      <c r="O36" s="8"/>
-      <c r="W36" s="11"/>
+      <c r="M36" s="4"/>
+      <c r="N36" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="O36" s="3"/>
+      <c r="P36" s="8"/>
       <c r="X36" s="11"/>
       <c r="Y36" s="11"/>
       <c r="Z36" s="11"/>
@@ -2293,8 +2342,9 @@
       <c r="AF36" s="11"/>
       <c r="AG36" s="11"/>
       <c r="AH36" s="11"/>
-    </row>
-    <row r="37" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI36" s="11"/>
+    </row>
+    <row r="37" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
         <v>20</v>
       </c>
@@ -2308,19 +2358,19 @@
         <v>136</v>
       </c>
       <c r="E37" s="29"/>
-      <c r="F37" s="2"/>
+      <c r="F37" s="44"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
-      <c r="J37" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K37" s="4"/>
+      <c r="J37" s="2"/>
+      <c r="K37" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L37" s="4"/>
-      <c r="M37" s="2"/>
-      <c r="N37" s="3"/>
-      <c r="O37" s="8"/>
-      <c r="W37" s="11"/>
+      <c r="M37" s="4"/>
+      <c r="N37" s="2"/>
+      <c r="O37" s="3"/>
+      <c r="P37" s="8"/>
       <c r="X37" s="11"/>
       <c r="Y37" s="11"/>
       <c r="Z37" s="11"/>
@@ -2332,8 +2382,9 @@
       <c r="AF37" s="11"/>
       <c r="AG37" s="11"/>
       <c r="AH37" s="11"/>
-    </row>
-    <row r="38" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI37" s="11"/>
+    </row>
+    <row r="38" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B38" s="9" t="s">
         <v>144</v>
       </c>
@@ -2344,17 +2395,17 @@
         <v>136</v>
       </c>
       <c r="E38" s="29"/>
-      <c r="F38" s="2"/>
+      <c r="F38" s="44"/>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
-      <c r="K38" s="4"/>
+      <c r="K38" s="2"/>
       <c r="L38" s="4"/>
-      <c r="M38" s="2"/>
-      <c r="N38" s="3"/>
-      <c r="O38" s="8"/>
-      <c r="W38" s="11"/>
+      <c r="M38" s="4"/>
+      <c r="N38" s="2"/>
+      <c r="O38" s="3"/>
+      <c r="P38" s="8"/>
       <c r="X38" s="11"/>
       <c r="Y38" s="11"/>
       <c r="Z38" s="11"/>
@@ -2366,8 +2417,9 @@
       <c r="AF38" s="11"/>
       <c r="AG38" s="11"/>
       <c r="AH38" s="11"/>
-    </row>
-    <row r="39" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI38" s="11"/>
+    </row>
+    <row r="39" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B39" s="9" t="s">
         <v>73</v>
       </c>
@@ -2378,17 +2430,17 @@
         <v>136</v>
       </c>
       <c r="E39" s="29"/>
-      <c r="F39" s="2"/>
+      <c r="F39" s="44"/>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
-      <c r="K39" s="4"/>
+      <c r="K39" s="2"/>
       <c r="L39" s="4"/>
-      <c r="M39" s="2"/>
-      <c r="N39" s="3"/>
-      <c r="O39" s="8"/>
-      <c r="W39" s="11"/>
+      <c r="M39" s="4"/>
+      <c r="N39" s="2"/>
+      <c r="O39" s="3"/>
+      <c r="P39" s="8"/>
       <c r="X39" s="11"/>
       <c r="Y39" s="11"/>
       <c r="Z39" s="11"/>
@@ -2399,8 +2451,9 @@
       <c r="AE39" s="11"/>
       <c r="AF39" s="11"/>
       <c r="AG39" s="11"/>
-    </row>
-    <row r="40" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AH39" s="11"/>
+    </row>
+    <row r="40" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B40" s="9" t="s">
         <v>74</v>
       </c>
@@ -2411,17 +2464,17 @@
         <v>136</v>
       </c>
       <c r="E40" s="29"/>
-      <c r="F40" s="2"/>
+      <c r="F40" s="44"/>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
-      <c r="K40" s="4"/>
+      <c r="K40" s="2"/>
       <c r="L40" s="4"/>
-      <c r="M40" s="2"/>
-      <c r="N40" s="3"/>
-      <c r="O40" s="8"/>
-      <c r="W40" s="11"/>
+      <c r="M40" s="4"/>
+      <c r="N40" s="2"/>
+      <c r="O40" s="3"/>
+      <c r="P40" s="8"/>
       <c r="X40" s="11"/>
       <c r="Y40" s="11"/>
       <c r="Z40" s="11"/>
@@ -2432,8 +2485,9 @@
       <c r="AE40" s="11"/>
       <c r="AF40" s="11"/>
       <c r="AG40" s="11"/>
-    </row>
-    <row r="41" spans="1:34" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="AH40" s="11"/>
+    </row>
+    <row r="41" spans="1:35" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="40" t="s">
         <v>116</v>
       </c>
@@ -2448,39 +2502,42 @@
         <v>30</v>
       </c>
       <c r="F41" s="16" t="s">
+        <v>145</v>
+      </c>
+      <c r="G41" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="G41" s="16" t="s">
+      <c r="H41" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="H41" s="16" t="s">
+      <c r="I41" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="I41" s="16" t="s">
+      <c r="J41" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="J41" s="16" t="s">
+      <c r="K41" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="K41" s="16" t="s">
+      <c r="L41" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="L41" s="16" t="s">
+      <c r="M41" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="M41" s="16" t="s">
+      <c r="N41" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="N41" s="16" t="s">
+      <c r="O41" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="O41" s="17" t="s">
+      <c r="P41" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="T41" s="11"/>
       <c r="U41" s="11"/>
-    </row>
-    <row r="42" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="V41" s="11"/>
+    </row>
+    <row r="42" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>120</v>
       </c>
@@ -2494,20 +2551,21 @@
         <v>125</v>
       </c>
       <c r="E42" s="30"/>
-      <c r="F42" s="7"/>
+      <c r="F42" s="45"/>
       <c r="G42" s="7"/>
       <c r="H42" s="7"/>
-      <c r="I42" s="2"/>
-      <c r="J42" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K42" s="2"/>
+      <c r="I42" s="7"/>
+      <c r="J42" s="2"/>
+      <c r="K42" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L42" s="2"/>
       <c r="M42" s="2"/>
-      <c r="N42" s="3"/>
+      <c r="N42" s="2"/>
       <c r="O42" s="3"/>
-    </row>
-    <row r="43" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P42" s="3"/>
+    </row>
+    <row r="43" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="22" t="s">
         <v>129</v>
@@ -2519,20 +2577,21 @@
         <v>130</v>
       </c>
       <c r="E43" s="30"/>
-      <c r="F43" s="7"/>
+      <c r="F43" s="45"/>
       <c r="G43" s="7"/>
       <c r="H43" s="7"/>
-      <c r="I43" s="2"/>
-      <c r="J43" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K43" s="2"/>
+      <c r="I43" s="7"/>
+      <c r="J43" s="2"/>
+      <c r="K43" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L43" s="2"/>
       <c r="M43" s="2"/>
-      <c r="N43" s="3"/>
+      <c r="N43" s="2"/>
       <c r="O43" s="3"/>
-    </row>
-    <row r="44" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="P43" s="3"/>
+    </row>
+    <row r="44" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A44" s="21" t="s">
         <v>121</v>
       </c>
@@ -2546,20 +2605,21 @@
         <v>126</v>
       </c>
       <c r="E44" s="30"/>
-      <c r="F44" s="7"/>
+      <c r="F44" s="45"/>
       <c r="G44" s="7"/>
       <c r="H44" s="7"/>
-      <c r="I44" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J44" s="2"/>
+      <c r="I44" s="7"/>
+      <c r="J44" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
       <c r="M44" s="2"/>
-      <c r="N44" s="3"/>
+      <c r="N44" s="2"/>
       <c r="O44" s="3"/>
-    </row>
-    <row r="45" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="P44" s="3"/>
+    </row>
+    <row r="45" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="22" t="s">
         <v>124</v>
@@ -2571,31 +2631,31 @@
         <v>126</v>
       </c>
       <c r="E45" s="30"/>
-      <c r="F45" s="7"/>
+      <c r="F45" s="45"/>
       <c r="G45" s="7"/>
       <c r="H45" s="7"/>
-      <c r="I45" s="2"/>
-      <c r="J45" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K45" s="2"/>
+      <c r="I45" s="7"/>
+      <c r="J45" s="2"/>
+      <c r="K45" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L45" s="2"/>
       <c r="M45" s="2"/>
-      <c r="N45" s="3"/>
+      <c r="N45" s="2"/>
       <c r="O45" s="3"/>
-      <c r="T45" s="11"/>
+      <c r="P45" s="3"/>
       <c r="U45" s="11"/>
-    </row>
-    <row r="50" spans="20:21" x14ac:dyDescent="0.25">
-      <c r="T50" s="11"/>
+      <c r="V45" s="11"/>
+    </row>
+    <row r="50" spans="21:22" x14ac:dyDescent="0.25">
       <c r="U50" s="11"/>
-    </row>
-    <row r="55" spans="20:21" x14ac:dyDescent="0.25">
-      <c r="T55" s="11"/>
+      <c r="V50" s="11"/>
+    </row>
+    <row r="55" spans="21:22" x14ac:dyDescent="0.25">
       <c r="U55" s="11"/>
-    </row>
-    <row r="72" spans="16:23" x14ac:dyDescent="0.25">
-      <c r="P72" s="11"/>
+      <c r="V55" s="11"/>
+    </row>
+    <row r="72" spans="17:24" x14ac:dyDescent="0.25">
       <c r="Q72" s="11"/>
       <c r="R72" s="11"/>
       <c r="S72" s="11"/>
@@ -2603,6 +2663,7 @@
       <c r="U72" s="11"/>
       <c r="V72" s="11"/>
       <c r="W72" s="11"/>
+      <c r="X72" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
marked all the tested commands
</commit_message>
<xml_diff>
--- a/8Bit Computer ver2.0/excel/commands.xlsx
+++ b/8Bit Computer ver2.0/excel/commands.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\8Bit_Computer\8Bit Computer ver2.0\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Files\GitHub\Computer_HTL\8Bit Computer ver2.0\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1819528-C0B5-4D8C-AA8A-DD4C33A17644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EB9D9BF-6474-493B-8011-387B7E3C8F44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3256ACAE-F419-450F-8F49-2183F1DCCADE}"/>
+    <workbookView xWindow="38550" yWindow="-2835" windowWidth="16410" windowHeight="18090" xr2:uid="{3256ACAE-F419-450F-8F49-2183F1DCCADE}"/>
   </bookViews>
   <sheets>
     <sheet name="Commands" sheetId="1" r:id="rId1"/>
@@ -20,9 +20,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -830,9 +827,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -851,9 +845,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1186,7 +1183,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02BDFC33-BE10-4835-94A0-E5C8BC037442}">
   <dimension ref="A1:AI72"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
     <col min="2" max="2" width="41.42578125" customWidth="1"/>
@@ -1206,10 +1203,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="1" customFormat="1" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="43"/>
+      <c r="B1" s="42"/>
       <c r="C1" s="16" t="s">
         <v>75</v>
       </c>
@@ -1323,7 +1320,7 @@
       <c r="E4" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="F4" s="39"/>
+      <c r="F4" s="32"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
@@ -1486,10 +1483,10 @@
       <c r="R9" s="1"/>
     </row>
     <row r="10" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="40" t="s">
+      <c r="A10" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="41"/>
+      <c r="B10" s="40"/>
       <c r="C10" s="16" t="s">
         <v>75</v>
       </c>
@@ -1681,7 +1678,7 @@
         <v>136</v>
       </c>
       <c r="E15" s="29"/>
-      <c r="F15" s="39"/>
+      <c r="F15" s="32"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2" t="s">
@@ -1716,7 +1713,7 @@
         <v>137</v>
       </c>
       <c r="E16" s="29"/>
-      <c r="F16" s="39"/>
+      <c r="F16" s="32"/>
       <c r="G16" s="2" t="s">
         <v>10</v>
       </c>
@@ -1840,7 +1837,7 @@
         <v>137</v>
       </c>
       <c r="E20" s="29"/>
-      <c r="F20" s="39"/>
+      <c r="F20" s="45"/>
       <c r="G20" s="2" t="s">
         <v>10</v>
       </c>
@@ -1967,7 +1964,7 @@
         <v>137</v>
       </c>
       <c r="E24" s="29"/>
-      <c r="F24" s="39"/>
+      <c r="F24" s="32"/>
       <c r="G24" s="2" t="s">
         <v>10</v>
       </c>
@@ -2029,7 +2026,7 @@
         <v>137</v>
       </c>
       <c r="E26" s="29"/>
-      <c r="F26" s="39"/>
+      <c r="F26" s="32"/>
       <c r="G26" s="2" t="s">
         <v>10</v>
       </c>
@@ -2088,7 +2085,7 @@
         <v>33</v>
       </c>
       <c r="E28" s="29"/>
-      <c r="F28" s="39"/>
+      <c r="F28" s="32"/>
       <c r="G28" s="2" t="s">
         <v>10</v>
       </c>
@@ -2226,7 +2223,7 @@
         <v>33</v>
       </c>
       <c r="E33" s="29"/>
-      <c r="F33" s="39"/>
+      <c r="F33" s="32"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
@@ -2253,7 +2250,7 @@
         <v>131</v>
       </c>
       <c r="E34" s="29"/>
-      <c r="F34" s="39"/>
+      <c r="F34" s="32"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
@@ -2280,7 +2277,7 @@
         <v>133</v>
       </c>
       <c r="E35" s="29"/>
-      <c r="F35" s="39"/>
+      <c r="F35" s="32"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
@@ -2319,7 +2316,7 @@
         <v>134</v>
       </c>
       <c r="E36" s="29"/>
-      <c r="F36" s="39"/>
+      <c r="F36" s="32"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
@@ -2467,7 +2464,7 @@
         <v>136</v>
       </c>
       <c r="E40" s="29"/>
-      <c r="F40" s="39"/>
+      <c r="F40" s="32"/>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
@@ -2491,10 +2488,10 @@
       <c r="AH40" s="11"/>
     </row>
     <row r="41" spans="1:35" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="42" t="s">
+      <c r="A41" s="41" t="s">
         <v>116</v>
       </c>
-      <c r="B41" s="43"/>
+      <c r="B41" s="42"/>
       <c r="C41" s="16" t="s">
         <v>75</v>
       </c>
@@ -2683,17 +2680,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9173A64-30DE-4BD7-9F06-BD4C8E1AFBD4}">
   <dimension ref="A2:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
     <col min="2" max="2" width="27.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="45"/>
+      <c r="B2" s="44"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -2740,10 +2737,10 @@
       </c>
     </row>
     <row r="13" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="44" t="s">
+      <c r="A13" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="45"/>
+      <c r="B13" s="44"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">

</xml_diff>

<commit_message>
worked on the test code
</commit_message>
<xml_diff>
--- a/8Bit Computer ver2.0/excel/commands.xlsx
+++ b/8Bit Computer ver2.0/excel/commands.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Files\GitHub\Computer_HTL\8Bit Computer ver2.0\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\8Bit_Computer\8Bit Computer ver2.0\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EB9D9BF-6474-493B-8011-387B7E3C8F44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC588BD4-C19A-400B-9001-FCD18CB452FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38550" yWindow="-2835" windowWidth="16410" windowHeight="18090" xr2:uid="{3256ACAE-F419-450F-8F49-2183F1DCCADE}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="14400" windowHeight="10665" xr2:uid="{3256ACAE-F419-450F-8F49-2183F1DCCADE}"/>
   </bookViews>
   <sheets>
     <sheet name="Commands" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,9 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -470,7 +473,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -729,7 +732,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -827,6 +830,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -845,12 +851,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1183,30 +1189,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02BDFC33-BE10-4835-94A0-E5C8BC037442}">
   <dimension ref="A1:AI72"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" customWidth="1"/>
-    <col min="2" max="2" width="41.42578125" customWidth="1"/>
-    <col min="3" max="3" width="8.42578125" customWidth="1"/>
-    <col min="4" max="5" width="12.140625" customWidth="1"/>
-    <col min="6" max="6" width="6.7109375" customWidth="1"/>
-    <col min="7" max="7" width="7.28515625" customWidth="1"/>
-    <col min="8" max="8" width="7.140625" customWidth="1"/>
-    <col min="9" max="9" width="7.42578125" customWidth="1"/>
-    <col min="10" max="10" width="10.85546875" customWidth="1"/>
+    <col min="1" max="1" width="15.75" customWidth="1"/>
+    <col min="2" max="2" width="41.375" customWidth="1"/>
+    <col min="3" max="3" width="8.375" customWidth="1"/>
+    <col min="4" max="5" width="12.125" customWidth="1"/>
+    <col min="6" max="6" width="6.75" customWidth="1"/>
+    <col min="7" max="7" width="7.25" customWidth="1"/>
+    <col min="8" max="8" width="7.125" customWidth="1"/>
+    <col min="9" max="9" width="7.375" customWidth="1"/>
+    <col min="10" max="10" width="10.875" customWidth="1"/>
     <col min="11" max="11" width="9" customWidth="1"/>
-    <col min="12" max="12" width="10.85546875" customWidth="1"/>
+    <col min="12" max="12" width="10.875" customWidth="1"/>
     <col min="13" max="13" width="9" customWidth="1"/>
     <col min="14" max="14" width="10" customWidth="1"/>
-    <col min="15" max="15" width="9.7109375" customWidth="1"/>
-    <col min="18" max="18" width="67.7109375" customWidth="1"/>
+    <col min="15" max="15" width="9.75" customWidth="1"/>
+    <col min="18" max="18" width="67.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="1" customFormat="1" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="41" t="s">
+    <row r="1" spans="1:18" s="1" customFormat="1" ht="18.75" thickBot="1">
+      <c r="A1" s="42" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="42"/>
+      <c r="B1" s="43"/>
       <c r="C1" s="16" t="s">
         <v>75</v>
       </c>
@@ -1250,7 +1256,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" s="1" customFormat="1">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1277,7 +1283,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18">
       <c r="B3" s="9" t="s">
         <v>59</v>
       </c>
@@ -1307,7 +1313,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="15" thickBot="1">
       <c r="B4" s="9" t="s">
         <v>58</v>
       </c>
@@ -1341,7 +1347,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18">
       <c r="A5" s="12" t="s">
         <v>127</v>
       </c>
@@ -1370,7 +1376,7 @@
       <c r="P5" s="1"/>
       <c r="R5" s="1"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18">
       <c r="B6" s="15" t="s">
         <v>114</v>
       </c>
@@ -1396,7 +1402,7 @@
       <c r="P6" s="1"/>
       <c r="R6" s="1"/>
     </row>
-    <row r="7" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" ht="15" thickBot="1">
       <c r="A7" s="19"/>
       <c r="B7" s="20" t="s">
         <v>115</v>
@@ -1423,7 +1429,7 @@
       <c r="P7" s="1"/>
       <c r="R7" s="1"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18">
       <c r="A8" s="12" t="s">
         <v>37</v>
       </c>
@@ -1454,7 +1460,7 @@
       <c r="P8" s="5"/>
       <c r="R8" s="1"/>
     </row>
-    <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" ht="15" thickBot="1">
       <c r="B9" s="15" t="s">
         <v>38</v>
       </c>
@@ -1482,11 +1488,11 @@
       <c r="P9" s="5"/>
       <c r="R9" s="1"/>
     </row>
-    <row r="10" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="39" t="s">
+    <row r="10" spans="1:18" ht="18.75" thickBot="1">
+      <c r="A10" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="40"/>
+      <c r="B10" s="41"/>
       <c r="C10" s="16" t="s">
         <v>75</v>
       </c>
@@ -1531,7 +1537,7 @@
       </c>
       <c r="R10" s="1"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -1566,7 +1572,7 @@
       <c r="P11" s="8"/>
       <c r="R11" s="1"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18">
       <c r="B12" s="9" t="s">
         <v>31</v>
       </c>
@@ -1600,7 +1606,7 @@
       <c r="P12" s="8"/>
       <c r="R12" s="1"/>
     </row>
-    <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="15" thickBot="1">
       <c r="B13" s="9" t="s">
         <v>5</v>
       </c>
@@ -1634,7 +1640,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18">
       <c r="A14" s="12" t="s">
         <v>40</v>
       </c>
@@ -1667,7 +1673,7 @@
       <c r="P14" s="8"/>
       <c r="R14" s="1"/>
     </row>
-    <row r="15" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" ht="15" thickBot="1">
       <c r="B15" s="10" t="s">
         <v>7</v>
       </c>
@@ -1699,7 +1705,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18">
       <c r="A16" s="12" t="s">
         <v>3</v>
       </c>
@@ -1732,7 +1738,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:22">
       <c r="B17" s="9" t="s">
         <v>22</v>
       </c>
@@ -1743,7 +1749,7 @@
         <v>137</v>
       </c>
       <c r="E17" s="29"/>
-      <c r="F17" s="4"/>
+      <c r="F17" s="46"/>
       <c r="G17" s="2" t="s">
         <v>10</v>
       </c>
@@ -1762,7 +1768,7 @@
       <c r="P17" s="8"/>
       <c r="R17" s="1"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:22">
       <c r="B18" s="9" t="s">
         <v>23</v>
       </c>
@@ -1773,7 +1779,7 @@
         <v>137</v>
       </c>
       <c r="E18" s="29"/>
-      <c r="F18" s="4"/>
+      <c r="F18" s="46"/>
       <c r="G18" s="2" t="s">
         <v>10</v>
       </c>
@@ -1794,7 +1800,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:22">
       <c r="B19" s="9" t="s">
         <v>24</v>
       </c>
@@ -1805,7 +1811,7 @@
         <v>137</v>
       </c>
       <c r="E19" s="29"/>
-      <c r="F19" s="4"/>
+      <c r="F19" s="46"/>
       <c r="G19" s="2" t="s">
         <v>10</v>
       </c>
@@ -1826,7 +1832,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:22">
       <c r="B20" s="9" t="s">
         <v>25</v>
       </c>
@@ -1837,7 +1843,7 @@
         <v>137</v>
       </c>
       <c r="E20" s="29"/>
-      <c r="F20" s="45"/>
+      <c r="F20" s="39"/>
       <c r="G20" s="2" t="s">
         <v>10</v>
       </c>
@@ -1856,7 +1862,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:22">
       <c r="B21" s="9" t="s">
         <v>26</v>
       </c>
@@ -1886,7 +1892,7 @@
       <c r="P21" s="8"/>
       <c r="R21" s="1"/>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:22">
       <c r="B22" s="9" t="s">
         <v>27</v>
       </c>
@@ -1918,7 +1924,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" ht="15" thickBot="1">
       <c r="B23" s="9" t="s">
         <v>28</v>
       </c>
@@ -1950,7 +1956,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:22">
       <c r="A24" s="12" t="s">
         <v>4</v>
       </c>
@@ -1984,7 +1990,7 @@
       </c>
       <c r="P24" s="8"/>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:22">
       <c r="B25" s="9" t="s">
         <v>47</v>
       </c>
@@ -2015,7 +2021,7 @@
       </c>
       <c r="P25" s="8"/>
     </row>
-    <row r="26" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:22" ht="15" thickBot="1">
       <c r="B26" s="9" t="s">
         <v>49</v>
       </c>
@@ -2046,7 +2052,7 @@
       </c>
       <c r="P26" s="8"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:22">
       <c r="A27" s="12" t="s">
         <v>112</v>
       </c>
@@ -2074,7 +2080,7 @@
       <c r="O27" s="3"/>
       <c r="P27" s="8"/>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:22">
       <c r="B28" s="9" t="s">
         <v>71</v>
       </c>
@@ -2101,7 +2107,7 @@
       <c r="O28" s="3"/>
       <c r="P28" s="8"/>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:22">
       <c r="B29" s="9" t="s">
         <v>65</v>
       </c>
@@ -2128,7 +2134,7 @@
       <c r="U29" s="11"/>
       <c r="V29" s="11"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:22">
       <c r="B30" s="9" t="s">
         <v>72</v>
       </c>
@@ -2139,7 +2145,7 @@
         <v>33</v>
       </c>
       <c r="E30" s="29"/>
-      <c r="F30" s="4"/>
+      <c r="F30" s="32"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2" t="s">
         <v>10</v>
@@ -2155,7 +2161,7 @@
       <c r="O30" s="3"/>
       <c r="P30" s="8"/>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:22">
       <c r="B31" s="15" t="s">
         <v>63</v>
       </c>
@@ -2180,7 +2186,7 @@
       <c r="O31" s="3"/>
       <c r="P31" s="8"/>
     </row>
-    <row r="32" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:22" ht="15" thickBot="1">
       <c r="B32" s="9" t="s">
         <v>69</v>
       </c>
@@ -2209,7 +2215,7 @@
       <c r="U32" s="11"/>
       <c r="V32" s="11"/>
     </row>
-    <row r="33" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:35">
       <c r="A33" s="12" t="s">
         <v>19</v>
       </c>
@@ -2239,7 +2245,7 @@
       </c>
       <c r="P33" s="8"/>
     </row>
-    <row r="34" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:35">
       <c r="B34" s="9" t="s">
         <v>67</v>
       </c>
@@ -2266,7 +2272,7 @@
       <c r="O34" s="3"/>
       <c r="P34" s="8"/>
     </row>
-    <row r="35" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:35">
       <c r="B35" s="9" t="s">
         <v>68</v>
       </c>
@@ -2305,7 +2311,7 @@
       <c r="AH35" s="11"/>
       <c r="AI35" s="11"/>
     </row>
-    <row r="36" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:35" ht="15" thickBot="1">
       <c r="B36" s="9" t="s">
         <v>8</v>
       </c>
@@ -2344,7 +2350,7 @@
       <c r="AH36" s="11"/>
       <c r="AI36" s="11"/>
     </row>
-    <row r="37" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:35">
       <c r="A37" s="12" t="s">
         <v>20</v>
       </c>
@@ -2384,7 +2390,7 @@
       <c r="AH37" s="11"/>
       <c r="AI37" s="11"/>
     </row>
-    <row r="38" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:35">
       <c r="B38" s="9" t="s">
         <v>144</v>
       </c>
@@ -2419,7 +2425,7 @@
       <c r="AH38" s="11"/>
       <c r="AI38" s="11"/>
     </row>
-    <row r="39" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:35">
       <c r="B39" s="9" t="s">
         <v>73</v>
       </c>
@@ -2453,7 +2459,7 @@
       <c r="AG39" s="11"/>
       <c r="AH39" s="11"/>
     </row>
-    <row r="40" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:35" ht="15" thickBot="1">
       <c r="B40" s="9" t="s">
         <v>74</v>
       </c>
@@ -2487,11 +2493,11 @@
       <c r="AG40" s="11"/>
       <c r="AH40" s="11"/>
     </row>
-    <row r="41" spans="1:35" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="41" t="s">
+    <row r="41" spans="1:35" ht="18.75" thickBot="1">
+      <c r="A41" s="42" t="s">
         <v>116</v>
       </c>
-      <c r="B41" s="42"/>
+      <c r="B41" s="43"/>
       <c r="C41" s="16" t="s">
         <v>75</v>
       </c>
@@ -2537,7 +2543,7 @@
       <c r="U41" s="11"/>
       <c r="V41" s="11"/>
     </row>
-    <row r="42" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:35">
       <c r="A42" s="1" t="s">
         <v>120</v>
       </c>
@@ -2565,7 +2571,7 @@
       <c r="O42" s="3"/>
       <c r="P42" s="3"/>
     </row>
-    <row r="43" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:35" ht="15" thickBot="1">
       <c r="A43" s="1"/>
       <c r="B43" s="22" t="s">
         <v>129</v>
@@ -2591,7 +2597,7 @@
       <c r="O43" s="3"/>
       <c r="P43" s="3"/>
     </row>
-    <row r="44" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:35">
       <c r="A44" s="21" t="s">
         <v>121</v>
       </c>
@@ -2619,7 +2625,7 @@
       <c r="O44" s="3"/>
       <c r="P44" s="3"/>
     </row>
-    <row r="45" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:35">
       <c r="A45" s="1"/>
       <c r="B45" s="22" t="s">
         <v>124</v>
@@ -2647,15 +2653,15 @@
       <c r="U45" s="11"/>
       <c r="V45" s="11"/>
     </row>
-    <row r="50" spans="21:22" x14ac:dyDescent="0.25">
+    <row r="50" spans="21:22">
       <c r="U50" s="11"/>
       <c r="V50" s="11"/>
     </row>
-    <row r="55" spans="21:22" x14ac:dyDescent="0.25">
+    <row r="55" spans="21:22">
       <c r="U55" s="11"/>
       <c r="V55" s="11"/>
     </row>
-    <row r="72" spans="17:24" x14ac:dyDescent="0.25">
+    <row r="72" spans="17:24">
       <c r="Q72" s="11"/>
       <c r="R72" s="11"/>
       <c r="S72" s="11"/>
@@ -2680,19 +2686,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9173A64-30DE-4BD7-9F06-BD4C8E1AFBD4}">
   <dimension ref="A2:B15"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.375" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" customWidth="1"/>
-    <col min="2" max="2" width="27.42578125" customWidth="1"/>
+    <col min="1" max="1" width="15.75" customWidth="1"/>
+    <col min="2" max="2" width="27.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="43" t="s">
+    <row r="2" spans="1:2" ht="18">
+      <c r="A2" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="44"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B2" s="45"/>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2700,12 +2706,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2">
       <c r="B4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -2713,12 +2719,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2">
       <c r="B7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>60</v>
       </c>
@@ -2726,23 +2732,23 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2">
       <c r="B10" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2">
       <c r="B11" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="43" t="s">
+    <row r="13" spans="1:2" ht="18">
+      <c r="A13" s="44" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="44"/>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13" s="45"/>
+    </row>
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>55</v>
       </c>
@@ -2750,7 +2756,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2">
       <c r="B15" t="s">
         <v>56</v>
       </c>

</xml_diff>

<commit_message>
worked on the test programme
still needs to be translated to hex, also still missing the input commands
</commit_message>
<xml_diff>
--- a/8Bit Computer ver2.0/excel/commands.xlsx
+++ b/8Bit Computer ver2.0/excel/commands.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\8Bit_Computer\8Bit Computer ver2.0\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Files\GitHub\Computer_HTL\8Bit Computer ver2.0\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC588BD4-C19A-400B-9001-FCD18CB452FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07858F00-B466-4C7E-8A1A-B0DFD7BDE014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="14400" windowHeight="10665" xr2:uid="{3256ACAE-F419-450F-8F49-2183F1DCCADE}"/>
+    <workbookView xWindow="27345" yWindow="900" windowWidth="11115" windowHeight="18585" xr2:uid="{3256ACAE-F419-450F-8F49-2183F1DCCADE}"/>
   </bookViews>
   <sheets>
     <sheet name="Commands" sheetId="1" r:id="rId1"/>
@@ -21,9 +21,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -473,7 +470,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -732,7 +729,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -830,7 +827,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -851,12 +848,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1189,26 +1183,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02BDFC33-BE10-4835-94A0-E5C8BC037442}">
   <dimension ref="A1:AI72"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.75" customWidth="1"/>
-    <col min="2" max="2" width="41.375" customWidth="1"/>
-    <col min="3" max="3" width="8.375" customWidth="1"/>
-    <col min="4" max="5" width="12.125" customWidth="1"/>
-    <col min="6" max="6" width="6.75" customWidth="1"/>
-    <col min="7" max="7" width="7.25" customWidth="1"/>
-    <col min="8" max="8" width="7.125" customWidth="1"/>
-    <col min="9" max="9" width="7.375" customWidth="1"/>
-    <col min="10" max="10" width="10.875" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="41.42578125" customWidth="1"/>
+    <col min="3" max="3" width="8.42578125" customWidth="1"/>
+    <col min="4" max="5" width="12.140625" customWidth="1"/>
+    <col min="6" max="6" width="6.7109375" customWidth="1"/>
+    <col min="7" max="7" width="7.28515625" customWidth="1"/>
+    <col min="8" max="8" width="7.140625" customWidth="1"/>
+    <col min="9" max="9" width="7.42578125" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" customWidth="1"/>
     <col min="11" max="11" width="9" customWidth="1"/>
-    <col min="12" max="12" width="10.875" customWidth="1"/>
+    <col min="12" max="12" width="10.85546875" customWidth="1"/>
     <col min="13" max="13" width="9" customWidth="1"/>
     <col min="14" max="14" width="10" customWidth="1"/>
-    <col min="15" max="15" width="9.75" customWidth="1"/>
-    <col min="18" max="18" width="67.75" customWidth="1"/>
+    <col min="15" max="15" width="9.7109375" customWidth="1"/>
+    <col min="18" max="18" width="67.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="1" customFormat="1" ht="18.75" thickBot="1">
+    <row r="1" spans="1:18" s="1" customFormat="1" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="42" t="s">
         <v>36</v>
       </c>
@@ -1256,7 +1250,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:18" s="1" customFormat="1">
+    <row r="2" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1283,7 +1277,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B3" s="9" t="s">
         <v>59</v>
       </c>
@@ -1313,7 +1307,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="15" thickBot="1">
+    <row r="4" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="9" t="s">
         <v>58</v>
       </c>
@@ -1347,7 +1341,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>127</v>
       </c>
@@ -1361,7 +1355,7 @@
         <v>33</v>
       </c>
       <c r="E5" s="34"/>
-      <c r="F5" s="4"/>
+      <c r="F5" s="39"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
       <c r="I5" s="7"/>
@@ -1376,7 +1370,7 @@
       <c r="P5" s="1"/>
       <c r="R5" s="1"/>
     </row>
-    <row r="6" spans="1:18">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B6" s="15" t="s">
         <v>114</v>
       </c>
@@ -1387,7 +1381,7 @@
         <v>33</v>
       </c>
       <c r="E6" s="34"/>
-      <c r="F6" s="4"/>
+      <c r="F6" s="39"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
@@ -1402,7 +1396,7 @@
       <c r="P6" s="1"/>
       <c r="R6" s="1"/>
     </row>
-    <row r="7" spans="1:18" ht="15" thickBot="1">
+    <row r="7" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="19"/>
       <c r="B7" s="20" t="s">
         <v>115</v>
@@ -1414,7 +1408,7 @@
       <c r="E7" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="F7" s="4"/>
+      <c r="F7" s="39"/>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
@@ -1429,7 +1423,7 @@
       <c r="P7" s="1"/>
       <c r="R7" s="1"/>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>37</v>
       </c>
@@ -1460,7 +1454,7 @@
       <c r="P8" s="5"/>
       <c r="R8" s="1"/>
     </row>
-    <row r="9" spans="1:18" ht="15" thickBot="1">
+    <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="15" t="s">
         <v>38</v>
       </c>
@@ -1488,7 +1482,7 @@
       <c r="P9" s="5"/>
       <c r="R9" s="1"/>
     </row>
-    <row r="10" spans="1:18" ht="18.75" thickBot="1">
+    <row r="10" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="40" t="s">
         <v>35</v>
       </c>
@@ -1537,7 +1531,7 @@
       </c>
       <c r="R10" s="1"/>
     </row>
-    <row r="11" spans="1:18">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -1572,7 +1566,7 @@
       <c r="P11" s="8"/>
       <c r="R11" s="1"/>
     </row>
-    <row r="12" spans="1:18">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B12" s="9" t="s">
         <v>31</v>
       </c>
@@ -1606,7 +1600,7 @@
       <c r="P12" s="8"/>
       <c r="R12" s="1"/>
     </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1">
+    <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="9" t="s">
         <v>5</v>
       </c>
@@ -1640,7 +1634,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:18">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
         <v>40</v>
       </c>
@@ -1673,7 +1667,7 @@
       <c r="P14" s="8"/>
       <c r="R14" s="1"/>
     </row>
-    <row r="15" spans="1:18" ht="15" thickBot="1">
+    <row r="15" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="10" t="s">
         <v>7</v>
       </c>
@@ -1705,7 +1699,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:18">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
         <v>3</v>
       </c>
@@ -1738,7 +1732,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:22">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B17" s="9" t="s">
         <v>22</v>
       </c>
@@ -1749,7 +1743,7 @@
         <v>137</v>
       </c>
       <c r="E17" s="29"/>
-      <c r="F17" s="46"/>
+      <c r="F17" s="39"/>
       <c r="G17" s="2" t="s">
         <v>10</v>
       </c>
@@ -1768,7 +1762,7 @@
       <c r="P17" s="8"/>
       <c r="R17" s="1"/>
     </row>
-    <row r="18" spans="1:22">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B18" s="9" t="s">
         <v>23</v>
       </c>
@@ -1779,7 +1773,7 @@
         <v>137</v>
       </c>
       <c r="E18" s="29"/>
-      <c r="F18" s="46"/>
+      <c r="F18" s="39"/>
       <c r="G18" s="2" t="s">
         <v>10</v>
       </c>
@@ -1800,7 +1794,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:22">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B19" s="9" t="s">
         <v>24</v>
       </c>
@@ -1811,7 +1805,7 @@
         <v>137</v>
       </c>
       <c r="E19" s="29"/>
-      <c r="F19" s="46"/>
+      <c r="F19" s="39"/>
       <c r="G19" s="2" t="s">
         <v>10</v>
       </c>
@@ -1832,7 +1826,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:22">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B20" s="9" t="s">
         <v>25</v>
       </c>
@@ -1862,7 +1856,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:22">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B21" s="9" t="s">
         <v>26</v>
       </c>
@@ -1873,7 +1867,7 @@
         <v>137</v>
       </c>
       <c r="E21" s="29"/>
-      <c r="F21" s="4"/>
+      <c r="F21" s="39"/>
       <c r="G21" s="2" t="s">
         <v>10</v>
       </c>
@@ -1892,7 +1886,7 @@
       <c r="P21" s="8"/>
       <c r="R21" s="1"/>
     </row>
-    <row r="22" spans="1:22">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B22" s="9" t="s">
         <v>27</v>
       </c>
@@ -1903,7 +1897,7 @@
         <v>137</v>
       </c>
       <c r="E22" s="29"/>
-      <c r="F22" s="4"/>
+      <c r="F22" s="39"/>
       <c r="G22" s="2" t="s">
         <v>10</v>
       </c>
@@ -1924,7 +1918,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:22" ht="15" thickBot="1">
+    <row r="23" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="9" t="s">
         <v>28</v>
       </c>
@@ -1935,7 +1929,7 @@
         <v>137</v>
       </c>
       <c r="E23" s="29"/>
-      <c r="F23" s="4"/>
+      <c r="F23" s="39"/>
       <c r="G23" s="2" t="s">
         <v>10</v>
       </c>
@@ -1956,7 +1950,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:22">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
         <v>4</v>
       </c>
@@ -1990,7 +1984,7 @@
       </c>
       <c r="P24" s="8"/>
     </row>
-    <row r="25" spans="1:22">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B25" s="9" t="s">
         <v>47</v>
       </c>
@@ -2021,7 +2015,7 @@
       </c>
       <c r="P25" s="8"/>
     </row>
-    <row r="26" spans="1:22" ht="15" thickBot="1">
+    <row r="26" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="9" t="s">
         <v>49</v>
       </c>
@@ -2052,7 +2046,7 @@
       </c>
       <c r="P26" s="8"/>
     </row>
-    <row r="27" spans="1:22">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
         <v>112</v>
       </c>
@@ -2080,7 +2074,7 @@
       <c r="O27" s="3"/>
       <c r="P27" s="8"/>
     </row>
-    <row r="28" spans="1:22">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B28" s="9" t="s">
         <v>71</v>
       </c>
@@ -2107,7 +2101,7 @@
       <c r="O28" s="3"/>
       <c r="P28" s="8"/>
     </row>
-    <row r="29" spans="1:22">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B29" s="9" t="s">
         <v>65</v>
       </c>
@@ -2134,7 +2128,7 @@
       <c r="U29" s="11"/>
       <c r="V29" s="11"/>
     </row>
-    <row r="30" spans="1:22">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B30" s="9" t="s">
         <v>72</v>
       </c>
@@ -2161,7 +2155,7 @@
       <c r="O30" s="3"/>
       <c r="P30" s="8"/>
     </row>
-    <row r="31" spans="1:22">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B31" s="15" t="s">
         <v>63</v>
       </c>
@@ -2186,7 +2180,7 @@
       <c r="O31" s="3"/>
       <c r="P31" s="8"/>
     </row>
-    <row r="32" spans="1:22" ht="15" thickBot="1">
+    <row r="32" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9" t="s">
         <v>69</v>
       </c>
@@ -2197,7 +2191,7 @@
         <v>33</v>
       </c>
       <c r="E32" s="29"/>
-      <c r="F32" s="4"/>
+      <c r="F32" s="39"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
       <c r="I32" s="2" t="s">
@@ -2215,7 +2209,7 @@
       <c r="U32" s="11"/>
       <c r="V32" s="11"/>
     </row>
-    <row r="33" spans="1:35">
+    <row r="33" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
         <v>19</v>
       </c>
@@ -2245,7 +2239,7 @@
       </c>
       <c r="P33" s="8"/>
     </row>
-    <row r="34" spans="1:35">
+    <row r="34" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B34" s="9" t="s">
         <v>67</v>
       </c>
@@ -2272,7 +2266,7 @@
       <c r="O34" s="3"/>
       <c r="P34" s="8"/>
     </row>
-    <row r="35" spans="1:35">
+    <row r="35" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B35" s="9" t="s">
         <v>68</v>
       </c>
@@ -2311,7 +2305,7 @@
       <c r="AH35" s="11"/>
       <c r="AI35" s="11"/>
     </row>
-    <row r="36" spans="1:35" ht="15" thickBot="1">
+    <row r="36" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="9" t="s">
         <v>8</v>
       </c>
@@ -2350,7 +2344,7 @@
       <c r="AH36" s="11"/>
       <c r="AI36" s="11"/>
     </row>
-    <row r="37" spans="1:35">
+    <row r="37" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
         <v>20</v>
       </c>
@@ -2390,7 +2384,7 @@
       <c r="AH37" s="11"/>
       <c r="AI37" s="11"/>
     </row>
-    <row r="38" spans="1:35">
+    <row r="38" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B38" s="9" t="s">
         <v>144</v>
       </c>
@@ -2401,7 +2395,7 @@
         <v>136</v>
       </c>
       <c r="E38" s="29"/>
-      <c r="F38" s="4"/>
+      <c r="F38" s="39"/>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
@@ -2425,7 +2419,7 @@
       <c r="AH38" s="11"/>
       <c r="AI38" s="11"/>
     </row>
-    <row r="39" spans="1:35">
+    <row r="39" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B39" s="9" t="s">
         <v>73</v>
       </c>
@@ -2459,7 +2453,7 @@
       <c r="AG39" s="11"/>
       <c r="AH39" s="11"/>
     </row>
-    <row r="40" spans="1:35" ht="15" thickBot="1">
+    <row r="40" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B40" s="9" t="s">
         <v>74</v>
       </c>
@@ -2493,7 +2487,7 @@
       <c r="AG40" s="11"/>
       <c r="AH40" s="11"/>
     </row>
-    <row r="41" spans="1:35" ht="18.75" thickBot="1">
+    <row r="41" spans="1:35" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="42" t="s">
         <v>116</v>
       </c>
@@ -2543,7 +2537,7 @@
       <c r="U41" s="11"/>
       <c r="V41" s="11"/>
     </row>
-    <row r="42" spans="1:35">
+    <row r="42" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>120</v>
       </c>
@@ -2571,7 +2565,7 @@
       <c r="O42" s="3"/>
       <c r="P42" s="3"/>
     </row>
-    <row r="43" spans="1:35" ht="15" thickBot="1">
+    <row r="43" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="22" t="s">
         <v>129</v>
@@ -2597,7 +2591,7 @@
       <c r="O43" s="3"/>
       <c r="P43" s="3"/>
     </row>
-    <row r="44" spans="1:35">
+    <row r="44" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A44" s="21" t="s">
         <v>121</v>
       </c>
@@ -2625,7 +2619,7 @@
       <c r="O44" s="3"/>
       <c r="P44" s="3"/>
     </row>
-    <row r="45" spans="1:35">
+    <row r="45" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="22" t="s">
         <v>124</v>
@@ -2637,7 +2631,7 @@
         <v>126</v>
       </c>
       <c r="E45" s="30"/>
-      <c r="F45" s="2"/>
+      <c r="F45" s="39"/>
       <c r="G45" s="7"/>
       <c r="H45" s="7"/>
       <c r="I45" s="7"/>
@@ -2653,15 +2647,15 @@
       <c r="U45" s="11"/>
       <c r="V45" s="11"/>
     </row>
-    <row r="50" spans="21:22">
+    <row r="50" spans="21:22" x14ac:dyDescent="0.25">
       <c r="U50" s="11"/>
       <c r="V50" s="11"/>
     </row>
-    <row r="55" spans="21:22">
+    <row r="55" spans="21:22" x14ac:dyDescent="0.25">
       <c r="U55" s="11"/>
       <c r="V55" s="11"/>
     </row>
-    <row r="72" spans="17:24">
+    <row r="72" spans="17:24" x14ac:dyDescent="0.25">
       <c r="Q72" s="11"/>
       <c r="R72" s="11"/>
       <c r="S72" s="11"/>
@@ -2686,19 +2680,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9173A64-30DE-4BD7-9F06-BD4C8E1AFBD4}">
   <dimension ref="A2:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.375" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.75" customWidth="1"/>
-    <col min="2" max="2" width="27.375" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2" ht="18">
+    <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A2" s="44" t="s">
         <v>35</v>
       </c>
       <c r="B2" s="45"/>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2706,12 +2700,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -2719,12 +2713,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>60</v>
       </c>
@@ -2732,23 +2726,23 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="18">
+    <row r="13" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A13" s="44" t="s">
         <v>36</v>
       </c>
       <c r="B13" s="45"/>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>55</v>
       </c>
@@ -2756,7 +2750,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>56</v>
       </c>

</xml_diff>

<commit_message>
added every command to the test
still needs translating and needs to be executed
</commit_message>
<xml_diff>
--- a/8Bit Computer ver2.0/excel/commands.xlsx
+++ b/8Bit Computer ver2.0/excel/commands.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Files\GitHub\Computer_HTL\8Bit Computer ver2.0\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07858F00-B466-4C7E-8A1A-B0DFD7BDE014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{762D9D55-268A-429A-9ED8-917376C9579A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="27345" yWindow="900" windowWidth="11115" windowHeight="18585" xr2:uid="{3256ACAE-F419-450F-8F49-2183F1DCCADE}"/>
   </bookViews>
@@ -2551,7 +2551,7 @@
         <v>125</v>
       </c>
       <c r="E42" s="30"/>
-      <c r="F42" s="2"/>
+      <c r="F42" s="39"/>
       <c r="G42" s="7"/>
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
@@ -2577,7 +2577,7 @@
         <v>130</v>
       </c>
       <c r="E43" s="30"/>
-      <c r="F43" s="2"/>
+      <c r="F43" s="39"/>
       <c r="G43" s="7"/>
       <c r="H43" s="7"/>
       <c r="I43" s="7"/>

</xml_diff>